<commit_message>
files: update Modeling_final.xlsx (Russ edits, pre-post version)
</commit_message>
<xml_diff>
--- a/2305/files/Modeling_final.xlsx
+++ b/2305/files/Modeling_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c6e3d429af62e1b5/ACC/2305/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rholl\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{778D0612-9C7D-4D44-9E98-809592764C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E4320A1-9D2C-47E3-9248-A86761EB014D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38299035-749A-4EEC-9E3D-858684E76C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-80" windowWidth="25820" windowHeight="14620" activeTab="4" xr2:uid="{86CF8DCD-D8AB-4717-BCE6-B8578E0C13DE}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{86CF8DCD-D8AB-4717-BCE6-B8578E0C13DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="2" r:id="rId1"/>
@@ -403,18 +403,18 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Thank you all for your contributions in class. I really hope this course wasn't too stressful. I've really been on a mission this semester to reimagine the curriculum in the courses I teach in a way that maximizes your vocational skill set. This sometimes means taking a lot of liberties with the tools and techniques I use to teach, and also means building the bridge as we drive over it. I hope I didn't stress you all out too much learning business statistics in fits and jerks; it certainly wasn't my intention to do so. 
+    <t>Of that 2025 ad spend  +8% , 60% will be spent evenly during the summer months: June, July, &amp; August</t>
+  </si>
+  <si>
+    <t>Perform a regression analysis (using the data analysis tool), and drop the output in cell i10. * remember to take note of decimals v percents</t>
+  </si>
+  <si>
+    <t>Student ID:</t>
+  </si>
+  <si>
+    <t>Thank you all for your contributions in class, I hope you picked up some good stuff along the way. I've designed this course to be a little different from the traditional curriculum, so I appreciate you all being flexible for how I teach. I hope I didn't overwhelm anyone, that was not my intention.
 What I did intend to do was communicate the elements of this course I know to be useful in the corporate world. I'd rather switch gears as many times as it takes if it means you know how to run a regression in Excel than to stick to the main line and drill y'all on equations because the book says so. I hope y'all got something out of it. I sure appreciate the opportunity to get y'all up to speed on the things I think will be valuable to you all in the future. Incidentally, I thought about letting you do some analysis on salaries with or without regression and correlation analysis, but opted out because it's a little self-serving, but I did include what I found below in case you need a reason to keep what you learned this spring fresh.
 I wish you all the best in your future endeavors. I'll be in touch if you ever have questions about the business world in Texas. If you don't mind, I'd also like to respectully ask for some feedback on the course. I'd love to hear anything you have for me on what were the high and low points, any advice for improving the curriculum, as well as advice for future students taking the course. Is the website good? Do y'all like the case studies? Is textbook optional a good idea? What would help make this class better. Thank you all in advance. Take care!</t>
-  </si>
-  <si>
-    <t>Of that 2025 ad spend  +8% , 60% will be spent evenly during the summer months: June, July, &amp; August</t>
-  </si>
-  <si>
-    <t>Perform a regression analysis (using the data analysis tool), and drop the output in cell i10. * remember to take note of decimals v percents</t>
-  </si>
-  <si>
-    <t>Student ID:</t>
   </si>
 </sst>
 </file>
@@ -809,10 +809,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1131,29 +1127,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E076F9DD-D273-41A6-960F-9805D5381293}">
   <dimension ref="B1:C6"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="3" width="67.1796875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.54296875" style="1"/>
+    <col min="3" max="3" width="67.19921875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.53125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B2" s="48" t="s">
         <v>71</v>
       </c>
       <c r="C2" s="50"/>
     </row>
-    <row r="3" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="4" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C4" s="50"/>
     </row>
-    <row r="6" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="3"/>
     </row>
   </sheetData>
@@ -1168,28 +1164,28 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A2:H66"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="6" max="6" width="84.54296875" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="72.453125" customWidth="1"/>
-    <col min="8" max="8" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.796875" customWidth="1"/>
+    <col min="4" max="4" width="15.19921875" customWidth="1"/>
+    <col min="6" max="6" width="84.53125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="72.46484375" customWidth="1"/>
+    <col min="8" max="8" width="24.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.45">
       <c r="F2" s="34" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="F3" s="35" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="2:7" collapsed="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" collapsed="1" x14ac:dyDescent="0.45">
       <c r="B7" s="6" t="s">
         <v>0</v>
       </c>
@@ -1206,7 +1202,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B8" s="26">
         <v>44957</v>
       </c>
@@ -1217,7 +1213,7 @@
         <v>17305</v>
       </c>
     </row>
-    <row r="9" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B9" s="26">
         <f>+EOMONTH(B8,1)</f>
         <v>44985</v>
@@ -1229,7 +1225,7 @@
         <v>20203</v>
       </c>
     </row>
-    <row r="10" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B10" s="26">
         <f t="shared" ref="B10:B43" si="0">+EOMONTH(B9,1)</f>
         <v>45016</v>
@@ -1241,7 +1237,7 @@
         <v>24213</v>
       </c>
     </row>
-    <row r="11" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B11" s="26">
         <f t="shared" si="0"/>
         <v>45046</v>
@@ -1253,7 +1249,7 @@
         <v>25955</v>
       </c>
     </row>
-    <row r="12" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B12" s="26">
         <f t="shared" si="0"/>
         <v>45077</v>
@@ -1265,7 +1261,7 @@
         <v>30333</v>
       </c>
     </row>
-    <row r="13" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B13" s="26">
         <f t="shared" si="0"/>
         <v>45107</v>
@@ -1277,7 +1273,7 @@
         <v>33132</v>
       </c>
     </row>
-    <row r="14" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B14" s="26">
         <f t="shared" si="0"/>
         <v>45138</v>
@@ -1289,7 +1285,7 @@
         <v>33346</v>
       </c>
     </row>
-    <row r="15" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B15" s="26">
         <f t="shared" si="0"/>
         <v>45169</v>
@@ -1301,7 +1297,7 @@
         <v>30632</v>
       </c>
     </row>
-    <row r="16" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B16" s="26">
         <f t="shared" si="0"/>
         <v>45199</v>
@@ -1313,7 +1309,7 @@
         <v>28121</v>
       </c>
     </row>
-    <row r="17" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B17" s="26">
         <f t="shared" si="0"/>
         <v>45230</v>
@@ -1325,7 +1321,7 @@
         <v>25241</v>
       </c>
     </row>
-    <row r="18" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B18" s="26">
         <f t="shared" si="0"/>
         <v>45260</v>
@@ -1337,7 +1333,7 @@
         <v>24257</v>
       </c>
     </row>
-    <row r="19" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B19" s="26">
         <f t="shared" si="0"/>
         <v>45291</v>
@@ -1349,7 +1345,7 @@
         <v>21313</v>
       </c>
     </row>
-    <row r="20" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B20" s="26">
         <f t="shared" si="0"/>
         <v>45322</v>
@@ -1361,7 +1357,7 @@
         <v>21156</v>
       </c>
     </row>
-    <row r="21" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B21" s="26">
         <f t="shared" si="0"/>
         <v>45351</v>
@@ -1373,7 +1369,7 @@
         <v>25883</v>
       </c>
     </row>
-    <row r="22" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B22" s="26">
         <f t="shared" si="0"/>
         <v>45382</v>
@@ -1385,7 +1381,7 @@
         <v>27880</v>
       </c>
     </row>
-    <row r="23" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B23" s="26">
         <f t="shared" si="0"/>
         <v>45412</v>
@@ -1397,7 +1393,7 @@
         <v>28602</v>
       </c>
     </row>
-    <row r="24" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B24" s="26">
         <f t="shared" si="0"/>
         <v>45443</v>
@@ -1409,7 +1405,7 @@
         <v>31903</v>
       </c>
     </row>
-    <row r="25" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B25" s="26">
         <f t="shared" si="0"/>
         <v>45473</v>
@@ -1421,7 +1417,7 @@
         <v>35018</v>
       </c>
     </row>
-    <row r="26" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B26" s="26">
         <f t="shared" si="0"/>
         <v>45504</v>
@@ -1433,7 +1429,7 @@
         <v>33465</v>
       </c>
     </row>
-    <row r="27" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B27" s="26">
         <f t="shared" si="0"/>
         <v>45535</v>
@@ -1445,7 +1441,7 @@
         <v>33757</v>
       </c>
     </row>
-    <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B28" s="26">
         <f t="shared" si="0"/>
         <v>45565</v>
@@ -1457,7 +1453,7 @@
         <v>30194</v>
       </c>
     </row>
-    <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B29" s="26">
         <f t="shared" si="0"/>
         <v>45596</v>
@@ -1469,7 +1465,7 @@
         <v>27020</v>
       </c>
     </row>
-    <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B30" s="26">
         <f t="shared" si="0"/>
         <v>45626</v>
@@ -1481,7 +1477,7 @@
         <v>26072</v>
       </c>
     </row>
-    <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B31" s="26">
         <f t="shared" si="0"/>
         <v>45657</v>
@@ -1493,7 +1489,7 @@
         <v>23849</v>
       </c>
     </row>
-    <row r="32" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B32" s="26">
         <f t="shared" si="0"/>
         <v>45688</v>
@@ -1505,7 +1501,7 @@
         <v>25510</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B33" s="26">
         <f t="shared" si="0"/>
         <v>45716</v>
@@ -1517,7 +1513,7 @@
         <v>26303</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B34" s="26">
         <f t="shared" si="0"/>
         <v>45747</v>
@@ -1529,7 +1525,7 @@
         <v>28284</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B35" s="26">
         <f t="shared" si="0"/>
         <v>45777</v>
@@ -1541,7 +1537,7 @@
         <v>32594</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B36" s="26">
         <f t="shared" si="0"/>
         <v>45808</v>
@@ -1553,7 +1549,7 @@
         <v>34601</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B37" s="26">
         <f t="shared" si="0"/>
         <v>45838</v>
@@ -1565,7 +1561,7 @@
         <v>35048</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B38" s="26">
         <f t="shared" si="0"/>
         <v>45869</v>
@@ -1577,7 +1573,7 @@
         <v>33679</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B39" s="26">
         <f t="shared" si="0"/>
         <v>45900</v>
@@ -1589,7 +1585,7 @@
         <v>35123</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.45">
       <c r="B40" s="26">
         <f t="shared" si="0"/>
         <v>45930</v>
@@ -1601,7 +1597,7 @@
         <v>33233</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="B41" s="26">
         <f t="shared" si="0"/>
         <v>45961</v>
@@ -1613,7 +1609,7 @@
         <v>28628</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="B42" s="26">
         <f t="shared" si="0"/>
         <v>45991</v>
@@ -1625,7 +1621,7 @@
         <v>26614</v>
       </c>
     </row>
-    <row r="43" spans="1:7" collapsed="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" collapsed="1" x14ac:dyDescent="0.45">
       <c r="A43" s="33" t="s">
         <v>39</v>
       </c>
@@ -1640,7 +1636,7 @@
         <v>26754</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="F44" s="29" t="s">
         <v>18</v>
       </c>
@@ -1648,7 +1644,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B45" s="26">
         <f>+EOMONTH(B43,1)</f>
         <v>46053</v>
@@ -1656,7 +1652,7 @@
       <c r="C45" s="31"/>
       <c r="D45" s="31"/>
     </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B46" s="26">
         <f t="shared" ref="B46:B56" si="1">+EOMONTH(B45,1)</f>
         <v>46081</v>
@@ -1668,7 +1664,7 @@
       </c>
       <c r="G46" s="24"/>
     </row>
-    <row r="47" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B47" s="26">
         <f t="shared" si="1"/>
         <v>46112</v>
@@ -1680,7 +1676,7 @@
       </c>
       <c r="G47" s="24"/>
     </row>
-    <row r="48" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B48" s="26">
         <f t="shared" si="1"/>
         <v>46142</v>
@@ -1692,7 +1688,7 @@
       </c>
       <c r="G48" s="24"/>
     </row>
-    <row r="49" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B49" s="26">
         <f t="shared" si="1"/>
         <v>46173</v>
@@ -1700,7 +1696,7 @@
       <c r="C49" s="31"/>
       <c r="D49" s="31"/>
     </row>
-    <row r="50" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B50" s="26">
         <f t="shared" si="1"/>
         <v>46203</v>
@@ -1712,7 +1708,7 @@
       </c>
       <c r="G50" s="25"/>
     </row>
-    <row r="51" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B51" s="26">
         <f t="shared" si="1"/>
         <v>46234</v>
@@ -1720,7 +1716,7 @@
       <c r="C51" s="31"/>
       <c r="D51" s="31"/>
     </row>
-    <row r="52" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B52" s="26">
         <f t="shared" si="1"/>
         <v>46265</v>
@@ -1735,7 +1731,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B53" s="26">
         <f t="shared" si="1"/>
         <v>46295</v>
@@ -1747,7 +1743,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B54" s="26">
         <f t="shared" si="1"/>
         <v>46326</v>
@@ -1755,7 +1751,7 @@
       <c r="C54" s="31"/>
       <c r="D54" s="31"/>
     </row>
-    <row r="55" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B55" s="26">
         <f t="shared" si="1"/>
         <v>46356</v>
@@ -1770,7 +1766,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B56" s="26">
         <f t="shared" si="1"/>
         <v>46387</v>
@@ -1778,7 +1774,7 @@
       <c r="C56" s="31"/>
       <c r="D56" s="31"/>
     </row>
-    <row r="57" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="F57" s="29" t="s">
         <v>27</v>
       </c>
@@ -1787,8 +1783,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="59" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="59" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="F59" s="29" t="s">
         <v>28</v>
       </c>
@@ -1797,25 +1793,25 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="62" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="62" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="F62" s="29" t="s">
         <v>30</v>
       </c>
       <c r="G62" s="27"/>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.45">
       <c r="F63" s="29" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.45">
       <c r="F64" s="29" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="6:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="66" spans="6:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="6:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="66" spans="6:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="F66" s="29" t="s">
         <v>32</v>
       </c>
@@ -1829,56 +1825,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33AF2F8-AD41-4565-840C-A969CF2888A6}">
   <dimension ref="A2:G207"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.46484375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41" customWidth="1"/>
-    <col min="3" max="3" width="32.54296875" style="15" customWidth="1"/>
+    <col min="3" max="3" width="32.53125" style="15" customWidth="1"/>
     <col min="4" max="4" width="22" style="15" customWidth="1"/>
-    <col min="6" max="6" width="91.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="91.53125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.46484375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.73046875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="12.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="F2" s="36" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="F3" s="35" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="F4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="F5" s="35" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="F6" s="35" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="F7" s="35"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="B8" s="8"/>
     </row>
-    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9" s="5" t="s">
         <v>73</v>
       </c>
@@ -1895,7 +1891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="9"/>
       <c r="B10" s="11">
         <v>46113</v>
@@ -1907,7 +1903,7 @@
       </c>
       <c r="G10" s="14"/>
     </row>
-    <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="9"/>
       <c r="B11" s="10">
         <v>46082</v>
@@ -1916,7 +1912,7 @@
       <c r="D11" s="54"/>
       <c r="G11" s="15"/>
     </row>
-    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" s="9"/>
       <c r="B12" s="11">
         <v>46054</v>
@@ -1928,7 +1924,7 @@
       </c>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A13" s="9"/>
       <c r="B13" s="10">
         <v>46023</v>
@@ -1936,7 +1932,7 @@
       <c r="C13" s="52"/>
       <c r="D13" s="54"/>
     </row>
-    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="9"/>
       <c r="B14" s="11">
         <v>45992</v>
@@ -1948,7 +1944,7 @@
       </c>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A15" s="9"/>
       <c r="B15" s="10">
         <v>45962</v>
@@ -1956,7 +1952,7 @@
       <c r="C15" s="52"/>
       <c r="D15" s="54"/>
     </row>
-    <row r="16" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A16" s="9"/>
       <c r="B16" s="11">
         <v>45931</v>
@@ -1968,7 +1964,7 @@
       </c>
       <c r="G16" s="13"/>
     </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A17" s="9"/>
       <c r="B17" s="10">
         <v>45901</v>
@@ -1976,7 +1972,7 @@
       <c r="C17" s="52"/>
       <c r="D17" s="54"/>
     </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A18" s="9"/>
       <c r="B18" s="11">
         <v>45870</v>
@@ -1988,7 +1984,7 @@
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="9"/>
       <c r="B19" s="10">
         <v>45839</v>
@@ -1996,7 +1992,7 @@
       <c r="C19" s="52"/>
       <c r="D19" s="54"/>
     </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="9"/>
       <c r="B20" s="11">
         <v>45809</v>
@@ -2008,7 +2004,7 @@
       </c>
       <c r="G20" s="16"/>
     </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="9"/>
       <c r="B21" s="10">
         <v>45778</v>
@@ -2016,7 +2012,7 @@
       <c r="C21" s="52"/>
       <c r="D21" s="54"/>
     </row>
-    <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="9"/>
       <c r="B22" s="11">
         <v>45748</v>
@@ -2028,7 +2024,7 @@
       </c>
       <c r="G22" s="16"/>
     </row>
-    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="9"/>
       <c r="B23" s="10">
         <v>45717</v>
@@ -2036,7 +2032,7 @@
       <c r="C23" s="52"/>
       <c r="D23" s="54"/>
     </row>
-    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A24" s="9"/>
       <c r="B24" s="11">
         <v>45689</v>
@@ -2048,7 +2044,7 @@
       </c>
       <c r="G24" s="16"/>
     </row>
-    <row r="25" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A25" s="9"/>
       <c r="B25" s="10">
         <v>45658</v>
@@ -2056,7 +2052,7 @@
       <c r="C25" s="52"/>
       <c r="D25" s="54"/>
     </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A26" s="9"/>
       <c r="B26" s="11">
         <v>45627</v>
@@ -2068,7 +2064,7 @@
       </c>
       <c r="G26" s="13"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="9"/>
       <c r="B27" s="10">
         <v>45597</v>
@@ -2076,7 +2072,7 @@
       <c r="C27" s="52"/>
       <c r="D27" s="54"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="9"/>
       <c r="B28" s="11">
         <v>45566</v>
@@ -2084,10 +2080,10 @@
       <c r="C28" s="51"/>
       <c r="D28" s="55"/>
       <c r="F28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="9"/>
       <c r="B29" s="10">
         <v>45536</v>
@@ -2095,7 +2091,7 @@
       <c r="C29" s="52"/>
       <c r="D29" s="54"/>
     </row>
-    <row r="30" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.45">
       <c r="A30" s="9"/>
       <c r="B30" s="11">
         <v>45505</v>
@@ -2106,7 +2102,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A31" s="9"/>
       <c r="B31" s="10">
         <v>45474</v>
@@ -2114,7 +2110,7 @@
       <c r="C31" s="52"/>
       <c r="D31" s="54"/>
     </row>
-    <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A32" s="9"/>
       <c r="B32" s="11">
         <v>45444</v>
@@ -2126,7 +2122,7 @@
       </c>
       <c r="G32" s="13"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="9"/>
       <c r="B33" s="10">
         <v>45413</v>
@@ -2134,7 +2130,7 @@
       <c r="C33" s="52"/>
       <c r="D33" s="54"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="9"/>
       <c r="B34" s="11">
         <v>45383</v>
@@ -2142,7 +2138,7 @@
       <c r="C34" s="51"/>
       <c r="D34" s="55"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="9"/>
       <c r="B35" s="10">
         <v>45352</v>
@@ -2150,7 +2146,7 @@
       <c r="C35" s="52"/>
       <c r="D35" s="54"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="9"/>
       <c r="B36" s="11">
         <v>45323</v>
@@ -2158,7 +2154,7 @@
       <c r="C36" s="51"/>
       <c r="D36" s="55"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="9"/>
       <c r="B37" s="10">
         <v>45292</v>
@@ -2166,7 +2162,7 @@
       <c r="C37" s="52"/>
       <c r="D37" s="54"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="9"/>
       <c r="B38" s="11">
         <v>45261</v>
@@ -2174,7 +2170,7 @@
       <c r="C38" s="51"/>
       <c r="D38" s="55"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="9"/>
       <c r="B39" s="10">
         <v>45231</v>
@@ -2182,7 +2178,7 @@
       <c r="C39" s="52"/>
       <c r="D39" s="54"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="9"/>
       <c r="B40" s="11">
         <v>45200</v>
@@ -2190,7 +2186,7 @@
       <c r="C40" s="51"/>
       <c r="D40" s="55"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="9"/>
       <c r="B41" s="10">
         <v>45170</v>
@@ -2198,7 +2194,7 @@
       <c r="C41" s="52"/>
       <c r="D41" s="54"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="9"/>
       <c r="B42" s="11">
         <v>45139</v>
@@ -2206,7 +2202,7 @@
       <c r="C42" s="51"/>
       <c r="D42" s="55"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" s="9"/>
       <c r="B43" s="10">
         <v>45108</v>
@@ -2214,7 +2210,7 @@
       <c r="C43" s="52"/>
       <c r="D43" s="54"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="9"/>
       <c r="B44" s="11">
         <v>45078</v>
@@ -2222,7 +2218,7 @@
       <c r="C44" s="51"/>
       <c r="D44" s="55"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" s="9"/>
       <c r="B45" s="10">
         <v>45047</v>
@@ -2230,7 +2226,7 @@
       <c r="C45" s="52"/>
       <c r="D45" s="54"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" s="9"/>
       <c r="B46" s="11">
         <v>45017</v>
@@ -2238,7 +2234,7 @@
       <c r="C46" s="51"/>
       <c r="D46" s="55"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" s="9"/>
       <c r="B47" s="10">
         <v>44986</v>
@@ -2246,7 +2242,7 @@
       <c r="C47" s="52"/>
       <c r="D47" s="54"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="9"/>
       <c r="B48" s="11">
         <v>44958</v>
@@ -2254,7 +2250,7 @@
       <c r="C48" s="51"/>
       <c r="D48" s="55"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="9"/>
       <c r="B49" s="10">
         <v>44927</v>
@@ -2262,7 +2258,7 @@
       <c r="C49" s="52"/>
       <c r="D49" s="54"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="9"/>
       <c r="B50" s="11">
         <v>44896</v>
@@ -2270,7 +2266,7 @@
       <c r="C50" s="51"/>
       <c r="D50" s="55"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A51" s="9"/>
       <c r="B51" s="10">
         <v>44866</v>
@@ -2278,7 +2274,7 @@
       <c r="C51" s="52"/>
       <c r="D51" s="54"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A52" s="9"/>
       <c r="B52" s="11">
         <v>44835</v>
@@ -2286,7 +2282,7 @@
       <c r="C52" s="51"/>
       <c r="D52" s="55"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A53" s="9"/>
       <c r="B53" s="10">
         <v>44805</v>
@@ -2294,7 +2290,7 @@
       <c r="C53" s="52"/>
       <c r="D53" s="54"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A54" s="9"/>
       <c r="B54" s="11">
         <v>44774</v>
@@ -2302,7 +2298,7 @@
       <c r="C54" s="51"/>
       <c r="D54" s="55"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A55" s="9"/>
       <c r="B55" s="10">
         <v>44743</v>
@@ -2310,7 +2306,7 @@
       <c r="C55" s="52"/>
       <c r="D55" s="54"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A56" s="9"/>
       <c r="B56" s="11">
         <v>44713</v>
@@ -2318,7 +2314,7 @@
       <c r="C56" s="51"/>
       <c r="D56" s="55"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A57" s="9"/>
       <c r="B57" s="10">
         <v>44682</v>
@@ -2326,7 +2322,7 @@
       <c r="C57" s="52"/>
       <c r="D57" s="54"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A58" s="9"/>
       <c r="B58" s="11">
         <v>44652</v>
@@ -2334,7 +2330,7 @@
       <c r="C58" s="51"/>
       <c r="D58" s="55"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A59" s="9"/>
       <c r="B59" s="10">
         <v>44621</v>
@@ -2342,7 +2338,7 @@
       <c r="C59" s="52"/>
       <c r="D59" s="54"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A60" s="9"/>
       <c r="B60" s="11">
         <v>44593</v>
@@ -2350,7 +2346,7 @@
       <c r="C60" s="51"/>
       <c r="D60" s="55"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A61" s="9"/>
       <c r="B61" s="10">
         <v>44562</v>
@@ -2358,7 +2354,7 @@
       <c r="C61" s="52"/>
       <c r="D61" s="54"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A62" s="9"/>
       <c r="B62" s="11">
         <v>44531</v>
@@ -2366,7 +2362,7 @@
       <c r="C62" s="51"/>
       <c r="D62" s="55"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A63" s="9"/>
       <c r="B63" s="10">
         <v>44501</v>
@@ -2374,7 +2370,7 @@
       <c r="C63" s="52"/>
       <c r="D63" s="54"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A64" s="9"/>
       <c r="B64" s="11">
         <v>44470</v>
@@ -2382,7 +2378,7 @@
       <c r="C64" s="51"/>
       <c r="D64" s="55"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A65" s="9"/>
       <c r="B65" s="10">
         <v>44440</v>
@@ -2390,7 +2386,7 @@
       <c r="C65" s="52"/>
       <c r="D65" s="54"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A66" s="9"/>
       <c r="B66" s="11">
         <v>44409</v>
@@ -2398,7 +2394,7 @@
       <c r="C66" s="51"/>
       <c r="D66" s="55"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A67" s="9"/>
       <c r="B67" s="10">
         <v>44378</v>
@@ -2406,7 +2402,7 @@
       <c r="C67" s="52"/>
       <c r="D67" s="54"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A68" s="9"/>
       <c r="B68" s="11">
         <v>44348</v>
@@ -2414,7 +2410,7 @@
       <c r="C68" s="51"/>
       <c r="D68" s="55"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A69" s="9"/>
       <c r="B69" s="10">
         <v>44317</v>
@@ -2422,7 +2418,7 @@
       <c r="C69" s="52"/>
       <c r="D69" s="54"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A70" s="9"/>
       <c r="B70" s="11">
         <v>44287</v>
@@ -2430,7 +2426,7 @@
       <c r="C70" s="51"/>
       <c r="D70" s="55"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A71" s="9"/>
       <c r="B71" s="10">
         <v>44256</v>
@@ -2438,7 +2434,7 @@
       <c r="C71" s="52"/>
       <c r="D71" s="54"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A72" s="9"/>
       <c r="B72" s="11">
         <v>44228</v>
@@ -2446,7 +2442,7 @@
       <c r="C72" s="51"/>
       <c r="D72" s="55"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A73" s="9"/>
       <c r="B73" s="10">
         <v>44197</v>
@@ -2454,7 +2450,7 @@
       <c r="C73" s="52"/>
       <c r="D73" s="54"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A74" s="9"/>
       <c r="B74" s="11">
         <v>44166</v>
@@ -2462,7 +2458,7 @@
       <c r="C74" s="51"/>
       <c r="D74" s="55"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A75" s="9"/>
       <c r="B75" s="10">
         <v>44136</v>
@@ -2470,7 +2466,7 @@
       <c r="C75" s="52"/>
       <c r="D75" s="54"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A76" s="9"/>
       <c r="B76" s="11">
         <v>44105</v>
@@ -2478,7 +2474,7 @@
       <c r="C76" s="51"/>
       <c r="D76" s="55"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A77" s="9"/>
       <c r="B77" s="10">
         <v>44075</v>
@@ -2486,7 +2482,7 @@
       <c r="C77" s="52"/>
       <c r="D77" s="54"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A78" s="9"/>
       <c r="B78" s="11">
         <v>44044</v>
@@ -2494,7 +2490,7 @@
       <c r="C78" s="51"/>
       <c r="D78" s="55"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A79" s="9"/>
       <c r="B79" s="10">
         <v>44013</v>
@@ -2502,7 +2498,7 @@
       <c r="C79" s="52"/>
       <c r="D79" s="54"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A80" s="9"/>
       <c r="B80" s="11">
         <v>43983</v>
@@ -2510,7 +2506,7 @@
       <c r="C80" s="51"/>
       <c r="D80" s="55"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A81" s="9"/>
       <c r="B81" s="10">
         <v>43952</v>
@@ -2518,7 +2514,7 @@
       <c r="C81" s="52"/>
       <c r="D81" s="54"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A82" s="9"/>
       <c r="B82" s="11">
         <v>43922</v>
@@ -2526,7 +2522,7 @@
       <c r="C82" s="51"/>
       <c r="D82" s="55"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A83" s="9"/>
       <c r="B83" s="10">
         <v>43891</v>
@@ -2534,7 +2530,7 @@
       <c r="C83" s="52"/>
       <c r="D83" s="54"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A84" s="9"/>
       <c r="B84" s="11">
         <v>43862</v>
@@ -2542,7 +2538,7 @@
       <c r="C84" s="51"/>
       <c r="D84" s="55"/>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A85" s="9"/>
       <c r="B85" s="10">
         <v>43831</v>
@@ -2550,7 +2546,7 @@
       <c r="C85" s="52"/>
       <c r="D85" s="54"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A86" s="9"/>
       <c r="B86" s="11">
         <v>43800</v>
@@ -2558,7 +2554,7 @@
       <c r="C86" s="51"/>
       <c r="D86" s="55"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A87" s="9"/>
       <c r="B87" s="10">
         <v>43770</v>
@@ -2566,7 +2562,7 @@
       <c r="C87" s="52"/>
       <c r="D87" s="54"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A88" s="9"/>
       <c r="B88" s="11">
         <v>43739</v>
@@ -2574,7 +2570,7 @@
       <c r="C88" s="51"/>
       <c r="D88" s="55"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A89" s="9"/>
       <c r="B89" s="10">
         <v>43709</v>
@@ -2582,7 +2578,7 @@
       <c r="C89" s="52"/>
       <c r="D89" s="54"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A90" s="9"/>
       <c r="B90" s="11">
         <v>43678</v>
@@ -2590,7 +2586,7 @@
       <c r="C90" s="51"/>
       <c r="D90" s="55"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A91" s="9"/>
       <c r="B91" s="10">
         <v>43647</v>
@@ -2598,7 +2594,7 @@
       <c r="C91" s="52"/>
       <c r="D91" s="54"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A92" s="9"/>
       <c r="B92" s="11">
         <v>43617</v>
@@ -2606,7 +2602,7 @@
       <c r="C92" s="51"/>
       <c r="D92" s="55"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A93" s="9"/>
       <c r="B93" s="10">
         <v>43586</v>
@@ -2614,7 +2610,7 @@
       <c r="C93" s="52"/>
       <c r="D93" s="54"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A94" s="9"/>
       <c r="B94" s="11">
         <v>43556</v>
@@ -2622,7 +2618,7 @@
       <c r="C94" s="51"/>
       <c r="D94" s="55"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A95" s="9"/>
       <c r="B95" s="10">
         <v>43525</v>
@@ -2630,7 +2626,7 @@
       <c r="C95" s="52"/>
       <c r="D95" s="54"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A96" s="9"/>
       <c r="B96" s="11">
         <v>43497</v>
@@ -2638,7 +2634,7 @@
       <c r="C96" s="51"/>
       <c r="D96" s="55"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A97" s="9"/>
       <c r="B97" s="10">
         <v>43466</v>
@@ -2646,7 +2642,7 @@
       <c r="C97" s="52"/>
       <c r="D97" s="54"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A98" s="9"/>
       <c r="B98" s="11">
         <v>43435</v>
@@ -2654,7 +2650,7 @@
       <c r="C98" s="51"/>
       <c r="D98" s="55"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A99" s="9"/>
       <c r="B99" s="10">
         <v>43405</v>
@@ -2662,7 +2658,7 @@
       <c r="C99" s="52"/>
       <c r="D99" s="54"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A100" s="9"/>
       <c r="B100" s="11">
         <v>43374</v>
@@ -2670,7 +2666,7 @@
       <c r="C100" s="51"/>
       <c r="D100" s="55"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A101" s="9"/>
       <c r="B101" s="10">
         <v>43344</v>
@@ -2678,7 +2674,7 @@
       <c r="C101" s="52"/>
       <c r="D101" s="54"/>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A102" s="9"/>
       <c r="B102" s="11">
         <v>43313</v>
@@ -2686,7 +2682,7 @@
       <c r="C102" s="51"/>
       <c r="D102" s="55"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A103" s="9"/>
       <c r="B103" s="10">
         <v>43282</v>
@@ -2694,7 +2690,7 @@
       <c r="C103" s="52"/>
       <c r="D103" s="54"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A104" s="9"/>
       <c r="B104" s="11">
         <v>43252</v>
@@ -2702,7 +2698,7 @@
       <c r="C104" s="51"/>
       <c r="D104" s="55"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A105" s="9"/>
       <c r="B105" s="10">
         <v>43221</v>
@@ -2710,7 +2706,7 @@
       <c r="C105" s="52"/>
       <c r="D105" s="54"/>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A106" s="9"/>
       <c r="B106" s="11">
         <v>43191</v>
@@ -2718,7 +2714,7 @@
       <c r="C106" s="51"/>
       <c r="D106" s="55"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A107" s="9"/>
       <c r="B107" s="10">
         <v>43160</v>
@@ -2726,7 +2722,7 @@
       <c r="C107" s="52"/>
       <c r="D107" s="54"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A108" s="9"/>
       <c r="B108" s="11">
         <v>43132</v>
@@ -2734,7 +2730,7 @@
       <c r="C108" s="51"/>
       <c r="D108" s="55"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A109" s="9"/>
       <c r="B109" s="10">
         <v>43101</v>
@@ -2742,7 +2738,7 @@
       <c r="C109" s="52"/>
       <c r="D109" s="54"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A110" s="9"/>
       <c r="B110" s="11">
         <v>43070</v>
@@ -2750,7 +2746,7 @@
       <c r="C110" s="51"/>
       <c r="D110" s="55"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A111" s="9"/>
       <c r="B111" s="10">
         <v>43040</v>
@@ -2758,7 +2754,7 @@
       <c r="C111" s="52"/>
       <c r="D111" s="54"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A112" s="9"/>
       <c r="B112" s="11">
         <v>43009</v>
@@ -2766,7 +2762,7 @@
       <c r="C112" s="51"/>
       <c r="D112" s="55"/>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A113" s="9"/>
       <c r="B113" s="10">
         <v>42979</v>
@@ -2774,7 +2770,7 @@
       <c r="C113" s="52"/>
       <c r="D113" s="54"/>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A114" s="9"/>
       <c r="B114" s="11">
         <v>42948</v>
@@ -2782,7 +2778,7 @@
       <c r="C114" s="51"/>
       <c r="D114" s="55"/>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A115" s="9"/>
       <c r="B115" s="10">
         <v>42917</v>
@@ -2790,7 +2786,7 @@
       <c r="C115" s="52"/>
       <c r="D115" s="54"/>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A116" s="9"/>
       <c r="B116" s="11">
         <v>42887</v>
@@ -2798,7 +2794,7 @@
       <c r="C116" s="51"/>
       <c r="D116" s="55"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A117" s="9"/>
       <c r="B117" s="10">
         <v>42856</v>
@@ -2806,7 +2802,7 @@
       <c r="C117" s="52"/>
       <c r="D117" s="54"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A118" s="9"/>
       <c r="B118" s="11">
         <v>42826</v>
@@ -2814,7 +2810,7 @@
       <c r="C118" s="51"/>
       <c r="D118" s="55"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A119" s="9"/>
       <c r="B119" s="10">
         <v>42795</v>
@@ -2822,7 +2818,7 @@
       <c r="C119" s="52"/>
       <c r="D119" s="54"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A120" s="9"/>
       <c r="B120" s="11">
         <v>42767</v>
@@ -2830,7 +2826,7 @@
       <c r="C120" s="51"/>
       <c r="D120" s="55"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A121" s="9"/>
       <c r="B121" s="10">
         <v>42736</v>
@@ -2838,7 +2834,7 @@
       <c r="C121" s="52"/>
       <c r="D121" s="54"/>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A122" s="9"/>
       <c r="B122" s="11">
         <v>42705</v>
@@ -2846,7 +2842,7 @@
       <c r="C122" s="51"/>
       <c r="D122" s="55"/>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A123" s="9"/>
       <c r="B123" s="10">
         <v>42675</v>
@@ -2854,7 +2850,7 @@
       <c r="C123" s="52"/>
       <c r="D123" s="54"/>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A124" s="9"/>
       <c r="B124" s="11">
         <v>42644</v>
@@ -2862,7 +2858,7 @@
       <c r="C124" s="51"/>
       <c r="D124" s="55"/>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A125" s="9"/>
       <c r="B125" s="10">
         <v>42614</v>
@@ -2870,7 +2866,7 @@
       <c r="C125" s="52"/>
       <c r="D125" s="54"/>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A126" s="9"/>
       <c r="B126" s="11">
         <v>42583</v>
@@ -2878,7 +2874,7 @@
       <c r="C126" s="51"/>
       <c r="D126" s="55"/>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A127" s="9"/>
       <c r="B127" s="10">
         <v>42552</v>
@@ -2886,7 +2882,7 @@
       <c r="C127" s="52"/>
       <c r="D127" s="54"/>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A128" s="9"/>
       <c r="B128" s="11">
         <v>42522</v>
@@ -2894,7 +2890,7 @@
       <c r="C128" s="51"/>
       <c r="D128" s="55"/>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A129" s="9"/>
       <c r="B129" s="10">
         <v>42491</v>
@@ -2902,7 +2898,7 @@
       <c r="C129" s="52"/>
       <c r="D129" s="54"/>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A130" s="9"/>
       <c r="B130" s="11">
         <v>42461</v>
@@ -2910,7 +2906,7 @@
       <c r="C130" s="51"/>
       <c r="D130" s="55"/>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A131" s="9"/>
       <c r="B131" s="10">
         <v>42430</v>
@@ -2918,7 +2914,7 @@
       <c r="C131" s="52"/>
       <c r="D131" s="54"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A132" s="9"/>
       <c r="B132" s="11">
         <v>42401</v>
@@ -2926,7 +2922,7 @@
       <c r="C132" s="51"/>
       <c r="D132" s="55"/>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A133" s="9"/>
       <c r="B133" s="10">
         <v>42370</v>
@@ -2934,7 +2930,7 @@
       <c r="C133" s="52"/>
       <c r="D133" s="54"/>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A134" s="9"/>
       <c r="B134" s="11">
         <v>42339</v>
@@ -2942,7 +2938,7 @@
       <c r="C134" s="51"/>
       <c r="D134" s="55"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A135" s="9"/>
       <c r="B135" s="10">
         <v>42309</v>
@@ -2950,7 +2946,7 @@
       <c r="C135" s="52"/>
       <c r="D135" s="54"/>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A136" s="9"/>
       <c r="B136" s="11">
         <v>42278</v>
@@ -2958,7 +2954,7 @@
       <c r="C136" s="51"/>
       <c r="D136" s="55"/>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A137" s="9"/>
       <c r="B137" s="10">
         <v>42248</v>
@@ -2966,7 +2962,7 @@
       <c r="C137" s="52"/>
       <c r="D137" s="54"/>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A138" s="9"/>
       <c r="B138" s="11">
         <v>42217</v>
@@ -2974,7 +2970,7 @@
       <c r="C138" s="51"/>
       <c r="D138" s="55"/>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A139" s="9"/>
       <c r="B139" s="10">
         <v>42186</v>
@@ -2982,7 +2978,7 @@
       <c r="C139" s="52"/>
       <c r="D139" s="54"/>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A140" s="9"/>
       <c r="B140" s="11">
         <v>42156</v>
@@ -2990,7 +2986,7 @@
       <c r="C140" s="51"/>
       <c r="D140" s="55"/>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A141" s="9"/>
       <c r="B141" s="10">
         <v>42125</v>
@@ -2998,7 +2994,7 @@
       <c r="C141" s="52"/>
       <c r="D141" s="54"/>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A142" s="9"/>
       <c r="B142" s="11">
         <v>42095</v>
@@ -3006,7 +3002,7 @@
       <c r="C142" s="51"/>
       <c r="D142" s="55"/>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A143" s="9"/>
       <c r="B143" s="10">
         <v>42064</v>
@@ -3014,7 +3010,7 @@
       <c r="C143" s="52"/>
       <c r="D143" s="54"/>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A144" s="9"/>
       <c r="B144" s="11">
         <v>42036</v>
@@ -3022,7 +3018,7 @@
       <c r="C144" s="51"/>
       <c r="D144" s="55"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A145" s="9"/>
       <c r="B145" s="10">
         <v>42005</v>
@@ -3030,7 +3026,7 @@
       <c r="C145" s="52"/>
       <c r="D145" s="54"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A146" s="9"/>
       <c r="B146" s="11">
         <v>41974</v>
@@ -3038,7 +3034,7 @@
       <c r="C146" s="51"/>
       <c r="D146" s="55"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A147" s="9"/>
       <c r="B147" s="10">
         <v>41944</v>
@@ -3046,7 +3042,7 @@
       <c r="C147" s="52"/>
       <c r="D147" s="54"/>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A148" s="9"/>
       <c r="B148" s="11">
         <v>41913</v>
@@ -3054,7 +3050,7 @@
       <c r="C148" s="51"/>
       <c r="D148" s="55"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A149" s="9"/>
       <c r="B149" s="10">
         <v>41883</v>
@@ -3062,7 +3058,7 @@
       <c r="C149" s="52"/>
       <c r="D149" s="54"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A150" s="9"/>
       <c r="B150" s="11">
         <v>41852</v>
@@ -3070,7 +3066,7 @@
       <c r="C150" s="51"/>
       <c r="D150" s="55"/>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A151" s="9"/>
       <c r="B151" s="10">
         <v>41821</v>
@@ -3078,7 +3074,7 @@
       <c r="C151" s="52"/>
       <c r="D151" s="54"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A152" s="9"/>
       <c r="B152" s="11">
         <v>41791</v>
@@ -3086,7 +3082,7 @@
       <c r="C152" s="51"/>
       <c r="D152" s="55"/>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A153" s="9"/>
       <c r="B153" s="10">
         <v>41760</v>
@@ -3094,7 +3090,7 @@
       <c r="C153" s="52"/>
       <c r="D153" s="54"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A154" s="9"/>
       <c r="B154" s="11">
         <v>41730</v>
@@ -3102,7 +3098,7 @@
       <c r="C154" s="51"/>
       <c r="D154" s="55"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A155" s="9"/>
       <c r="B155" s="10">
         <v>41699</v>
@@ -3110,7 +3106,7 @@
       <c r="C155" s="52"/>
       <c r="D155" s="54"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A156" s="9"/>
       <c r="B156" s="11">
         <v>41671</v>
@@ -3118,7 +3114,7 @@
       <c r="C156" s="51"/>
       <c r="D156" s="55"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A157" s="9"/>
       <c r="B157" s="10">
         <v>41640</v>
@@ -3126,7 +3122,7 @@
       <c r="C157" s="52"/>
       <c r="D157" s="54"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A158" s="9"/>
       <c r="B158" s="11">
         <v>41609</v>
@@ -3134,7 +3130,7 @@
       <c r="C158" s="51"/>
       <c r="D158" s="55"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A159" s="9"/>
       <c r="B159" s="10">
         <v>41579</v>
@@ -3142,7 +3138,7 @@
       <c r="C159" s="52"/>
       <c r="D159" s="54"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A160" s="9"/>
       <c r="B160" s="11">
         <v>41548</v>
@@ -3150,7 +3146,7 @@
       <c r="C160" s="51"/>
       <c r="D160" s="55"/>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A161" s="9"/>
       <c r="B161" s="10">
         <v>41518</v>
@@ -3158,7 +3154,7 @@
       <c r="C161" s="52"/>
       <c r="D161" s="54"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A162" s="9"/>
       <c r="B162" s="11">
         <v>41487</v>
@@ -3166,7 +3162,7 @@
       <c r="C162" s="51"/>
       <c r="D162" s="55"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A163" s="9"/>
       <c r="B163" s="10">
         <v>41456</v>
@@ -3174,7 +3170,7 @@
       <c r="C163" s="52"/>
       <c r="D163" s="54"/>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A164" s="9"/>
       <c r="B164" s="11">
         <v>41426</v>
@@ -3182,7 +3178,7 @@
       <c r="C164" s="51"/>
       <c r="D164" s="55"/>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A165" s="9"/>
       <c r="B165" s="10">
         <v>41395</v>
@@ -3190,7 +3186,7 @@
       <c r="C165" s="52"/>
       <c r="D165" s="54"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A166" s="9"/>
       <c r="B166" s="11">
         <v>41365</v>
@@ -3198,7 +3194,7 @@
       <c r="C166" s="51"/>
       <c r="D166" s="55"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A167" s="9"/>
       <c r="B167" s="10">
         <v>41334</v>
@@ -3206,7 +3202,7 @@
       <c r="C167" s="52"/>
       <c r="D167" s="54"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A168" s="9"/>
       <c r="B168" s="11">
         <v>41306</v>
@@ -3214,7 +3210,7 @@
       <c r="C168" s="51"/>
       <c r="D168" s="55"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A169" s="9"/>
       <c r="B169" s="10">
         <v>41275</v>
@@ -3222,7 +3218,7 @@
       <c r="C169" s="52"/>
       <c r="D169" s="54"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A170" s="9"/>
       <c r="B170" s="11">
         <v>41244</v>
@@ -3230,7 +3226,7 @@
       <c r="C170" s="51"/>
       <c r="D170" s="55"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A171" s="9"/>
       <c r="B171" s="10">
         <v>41214</v>
@@ -3238,7 +3234,7 @@
       <c r="C171" s="52"/>
       <c r="D171" s="54"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A172" s="9"/>
       <c r="B172" s="11">
         <v>41183</v>
@@ -3246,7 +3242,7 @@
       <c r="C172" s="51"/>
       <c r="D172" s="55"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A173" s="9"/>
       <c r="B173" s="10">
         <v>41153</v>
@@ -3254,7 +3250,7 @@
       <c r="C173" s="52"/>
       <c r="D173" s="54"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A174" s="9"/>
       <c r="B174" s="11">
         <v>41122</v>
@@ -3262,7 +3258,7 @@
       <c r="C174" s="51"/>
       <c r="D174" s="55"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A175" s="9"/>
       <c r="B175" s="10">
         <v>41091</v>
@@ -3270,7 +3266,7 @@
       <c r="C175" s="52"/>
       <c r="D175" s="54"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A176" s="9"/>
       <c r="B176" s="11">
         <v>41061</v>
@@ -3278,7 +3274,7 @@
       <c r="C176" s="51"/>
       <c r="D176" s="55"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A177" s="9"/>
       <c r="B177" s="10">
         <v>41030</v>
@@ -3286,7 +3282,7 @@
       <c r="C177" s="52"/>
       <c r="D177" s="54"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A178" s="9"/>
       <c r="B178" s="11">
         <v>41000</v>
@@ -3294,7 +3290,7 @@
       <c r="C178" s="51"/>
       <c r="D178" s="55"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A179" s="9"/>
       <c r="B179" s="10">
         <v>40969</v>
@@ -3302,7 +3298,7 @@
       <c r="C179" s="52"/>
       <c r="D179" s="54"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A180" s="9"/>
       <c r="B180" s="11">
         <v>40940</v>
@@ -3310,7 +3306,7 @@
       <c r="C180" s="51"/>
       <c r="D180" s="55"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A181" s="9"/>
       <c r="B181" s="10">
         <v>40909</v>
@@ -3318,7 +3314,7 @@
       <c r="C181" s="52"/>
       <c r="D181" s="54"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A182" s="9"/>
       <c r="B182" s="11">
         <v>40878</v>
@@ -3326,7 +3322,7 @@
       <c r="C182" s="51"/>
       <c r="D182" s="55"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A183" s="9"/>
       <c r="B183" s="10">
         <v>40848</v>
@@ -3334,7 +3330,7 @@
       <c r="C183" s="52"/>
       <c r="D183" s="54"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A184" s="9"/>
       <c r="B184" s="11">
         <v>40817</v>
@@ -3342,7 +3338,7 @@
       <c r="C184" s="51"/>
       <c r="D184" s="55"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A185" s="9"/>
       <c r="B185" s="10">
         <v>40787</v>
@@ -3350,7 +3346,7 @@
       <c r="C185" s="52"/>
       <c r="D185" s="54"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A186" s="9"/>
       <c r="B186" s="11">
         <v>40756</v>
@@ -3358,7 +3354,7 @@
       <c r="C186" s="51"/>
       <c r="D186" s="55"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A187" s="9"/>
       <c r="B187" s="10">
         <v>40725</v>
@@ -3366,7 +3362,7 @@
       <c r="C187" s="52"/>
       <c r="D187" s="54"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A188" s="9"/>
       <c r="B188" s="11">
         <v>40695</v>
@@ -3374,7 +3370,7 @@
       <c r="C188" s="51"/>
       <c r="D188" s="55"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A189" s="9"/>
       <c r="B189" s="10">
         <v>40664</v>
@@ -3382,7 +3378,7 @@
       <c r="C189" s="52"/>
       <c r="D189" s="54"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A190" s="9"/>
       <c r="B190" s="11">
         <v>40634</v>
@@ -3390,7 +3386,7 @@
       <c r="C190" s="51"/>
       <c r="D190" s="55"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A191" s="9"/>
       <c r="B191" s="10">
         <v>40603</v>
@@ -3398,7 +3394,7 @@
       <c r="C191" s="52"/>
       <c r="D191" s="54"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A192" s="9"/>
       <c r="B192" s="11">
         <v>40575</v>
@@ -3406,7 +3402,7 @@
       <c r="C192" s="51"/>
       <c r="D192" s="55"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A193" s="9"/>
       <c r="B193" s="10">
         <v>40544</v>
@@ -3414,7 +3410,7 @@
       <c r="C193" s="52"/>
       <c r="D193" s="54"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A194" s="9"/>
       <c r="B194" s="11">
         <v>40513</v>
@@ -3422,7 +3418,7 @@
       <c r="C194" s="51"/>
       <c r="D194" s="55"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A195" s="9"/>
       <c r="B195" s="10">
         <v>40483</v>
@@ -3430,7 +3426,7 @@
       <c r="C195" s="52"/>
       <c r="D195" s="54"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A196" s="9"/>
       <c r="B196" s="11">
         <v>40452</v>
@@ -3438,7 +3434,7 @@
       <c r="C196" s="51"/>
       <c r="D196" s="55"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A197" s="9"/>
       <c r="B197" s="10">
         <v>40422</v>
@@ -3446,7 +3442,7 @@
       <c r="C197" s="52"/>
       <c r="D197" s="54"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A198" s="9"/>
       <c r="B198" s="11">
         <v>40391</v>
@@ -3454,7 +3450,7 @@
       <c r="C198" s="51"/>
       <c r="D198" s="55"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A199" s="9"/>
       <c r="B199" s="10">
         <v>40360</v>
@@ -3462,7 +3458,7 @@
       <c r="C199" s="52"/>
       <c r="D199" s="54"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A200" s="9"/>
       <c r="B200" s="11">
         <v>40330</v>
@@ -3470,7 +3466,7 @@
       <c r="C200" s="51"/>
       <c r="D200" s="55"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A201" s="9"/>
       <c r="B201" s="10">
         <v>40299</v>
@@ -3478,7 +3474,7 @@
       <c r="C201" s="52"/>
       <c r="D201" s="54"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A202" s="9"/>
       <c r="B202" s="11">
         <v>40269</v>
@@ -3486,7 +3482,7 @@
       <c r="C202" s="51"/>
       <c r="D202" s="55"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A203" s="9"/>
       <c r="B203" s="10">
         <v>40238</v>
@@ -3494,7 +3490,7 @@
       <c r="C203" s="52"/>
       <c r="D203" s="54"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A204" s="9"/>
       <c r="B204" s="11">
         <v>40210</v>
@@ -3502,7 +3498,7 @@
       <c r="C204" s="51"/>
       <c r="D204" s="55"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A205" s="9"/>
       <c r="B205" s="10">
         <v>40179</v>
@@ -3510,7 +3506,7 @@
       <c r="C205" s="52"/>
       <c r="D205" s="54"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B207" s="4" t="s">
         <v>5</v>
       </c>
@@ -3528,31 +3524,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3A9E5C-C640-4448-9A91-F1BC9187C7A3}">
   <dimension ref="B2:J106"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="2" max="2" width="18.796875" customWidth="1"/>
     <col min="3" max="3" width="17" style="20" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" style="20" customWidth="1"/>
-    <col min="5" max="5" width="26.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.46484375" style="20" customWidth="1"/>
+    <col min="5" max="5" width="26.46484375" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="5.26953125" customWidth="1"/>
-    <col min="8" max="8" width="82.7265625" style="40" customWidth="1"/>
-    <col min="9" max="9" width="35.453125" style="40" customWidth="1"/>
-    <col min="10" max="10" width="12.7265625" style="57" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.265625" customWidth="1"/>
+    <col min="8" max="8" width="82.73046875" style="40" customWidth="1"/>
+    <col min="9" max="9" width="35.46484375" style="40" customWidth="1"/>
+    <col min="10" max="10" width="12.73046875" style="57" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.73046875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="12.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" ht="57" x14ac:dyDescent="0.45">
       <c r="H2" s="39" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:9" ht="15.75" x14ac:dyDescent="0.45">
       <c r="B6" s="18" t="s">
         <v>43</v>
       </c>
@@ -3575,7 +3571,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B7">
         <v>1</v>
       </c>
@@ -3595,7 +3591,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8">
         <v>2</v>
       </c>
@@ -3612,7 +3608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9">
         <v>3</v>
       </c>
@@ -3633,7 +3629,7 @@
       </c>
       <c r="I9" s="42"/>
     </row>
-    <row r="10" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B10">
         <v>4</v>
       </c>
@@ -3654,7 +3650,7 @@
       </c>
       <c r="I10" s="42"/>
     </row>
-    <row r="11" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11">
         <v>5</v>
       </c>
@@ -3675,7 +3671,7 @@
       </c>
       <c r="I11" s="42"/>
     </row>
-    <row r="12" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12">
         <v>6</v>
       </c>
@@ -3692,7 +3688,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B13">
         <v>7</v>
       </c>
@@ -3713,7 +3709,7 @@
       </c>
       <c r="I13" s="56"/>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B14">
         <v>8</v>
       </c>
@@ -3730,7 +3726,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B15">
         <v>9</v>
       </c>
@@ -3747,7 +3743,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B16">
         <v>10</v>
       </c>
@@ -3767,7 +3763,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B17">
         <v>11</v>
       </c>
@@ -3787,7 +3783,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18">
         <v>12</v>
       </c>
@@ -3804,7 +3800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19">
         <v>13</v>
       </c>
@@ -3825,7 +3821,7 @@
       </c>
       <c r="I19" s="43"/>
     </row>
-    <row r="20" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B20">
         <v>14</v>
       </c>
@@ -3846,7 +3842,7 @@
       </c>
       <c r="I20" s="43"/>
     </row>
-    <row r="21" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B21">
         <v>15</v>
       </c>
@@ -3867,7 +3863,7 @@
       </c>
       <c r="I21" s="43"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B22">
         <v>16</v>
       </c>
@@ -3884,7 +3880,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B23">
         <v>17</v>
       </c>
@@ -3905,7 +3901,7 @@
       </c>
       <c r="I23" s="12"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B24">
         <v>18</v>
       </c>
@@ -3922,7 +3918,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B25">
         <v>19</v>
       </c>
@@ -3942,7 +3938,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B26">
         <v>20</v>
       </c>
@@ -3959,7 +3955,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B27">
         <v>21</v>
       </c>
@@ -3979,7 +3975,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B28">
         <v>22</v>
       </c>
@@ -3996,7 +3992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B29">
         <v>23</v>
       </c>
@@ -4020,7 +4016,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B30">
         <v>24</v>
       </c>
@@ -4037,7 +4033,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:10" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:10" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B31">
         <v>25</v>
       </c>
@@ -4061,7 +4057,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B32">
         <v>26</v>
       </c>
@@ -4078,7 +4074,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B33">
         <v>27</v>
       </c>
@@ -4095,7 +4091,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="2:10" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="2:10" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B34">
         <v>28</v>
       </c>
@@ -4119,7 +4115,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B35">
         <v>29</v>
       </c>
@@ -4136,7 +4132,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B36">
         <v>30</v>
       </c>
@@ -4156,7 +4152,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="37" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B37">
         <v>31</v>
       </c>
@@ -4173,7 +4169,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B38">
         <v>32</v>
       </c>
@@ -4197,7 +4193,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="39" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B39">
         <v>33</v>
       </c>
@@ -4214,7 +4210,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:10" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="2:10" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B40">
         <v>34</v>
       </c>
@@ -4238,7 +4234,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B41">
         <v>35</v>
       </c>
@@ -4255,7 +4251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B42">
         <v>36</v>
       </c>
@@ -4272,7 +4268,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B43">
         <v>37</v>
       </c>
@@ -4289,7 +4285,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B44">
         <v>38</v>
       </c>
@@ -4306,7 +4302,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B45">
         <v>39</v>
       </c>
@@ -4323,7 +4319,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B46">
         <v>40</v>
       </c>
@@ -4340,7 +4336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B47">
         <v>41</v>
       </c>
@@ -4357,7 +4353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B48">
         <v>42</v>
       </c>
@@ -4374,7 +4370,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B49">
         <v>43</v>
       </c>
@@ -4391,7 +4387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B50">
         <v>44</v>
       </c>
@@ -4408,7 +4404,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B51">
         <v>45</v>
       </c>
@@ -4425,7 +4421,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B52">
         <v>46</v>
       </c>
@@ -4442,7 +4438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B53">
         <v>47</v>
       </c>
@@ -4459,7 +4455,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B54">
         <v>48</v>
       </c>
@@ -4476,7 +4472,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B55">
         <v>49</v>
       </c>
@@ -4493,7 +4489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B56">
         <v>50</v>
       </c>
@@ -4510,7 +4506,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B57">
         <v>51</v>
       </c>
@@ -4527,7 +4523,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B58">
         <v>52</v>
       </c>
@@ -4544,7 +4540,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B59">
         <v>53</v>
       </c>
@@ -4561,7 +4557,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B60">
         <v>54</v>
       </c>
@@ -4578,7 +4574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B61">
         <v>55</v>
       </c>
@@ -4595,7 +4591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B62">
         <v>56</v>
       </c>
@@ -4612,7 +4608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B63">
         <v>57</v>
       </c>
@@ -4629,7 +4625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B64">
         <v>58</v>
       </c>
@@ -4646,7 +4642,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B65">
         <v>59</v>
       </c>
@@ -4663,7 +4659,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B66">
         <v>60</v>
       </c>
@@ -4680,7 +4676,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B67">
         <v>61</v>
       </c>
@@ -4697,7 +4693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B68">
         <v>62</v>
       </c>
@@ -4714,7 +4710,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B69">
         <v>63</v>
       </c>
@@ -4731,7 +4727,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B70">
         <v>64</v>
       </c>
@@ -4748,7 +4744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B71">
         <v>65</v>
       </c>
@@ -4765,7 +4761,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B72">
         <v>66</v>
       </c>
@@ -4782,7 +4778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B73">
         <v>67</v>
       </c>
@@ -4799,7 +4795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B74">
         <v>68</v>
       </c>
@@ -4816,7 +4812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B75">
         <v>69</v>
       </c>
@@ -4833,7 +4829,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B76">
         <v>70</v>
       </c>
@@ -4850,7 +4846,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B77">
         <v>71</v>
       </c>
@@ -4867,7 +4863,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B78">
         <v>72</v>
       </c>
@@ -4884,7 +4880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B79">
         <v>73</v>
       </c>
@@ -4901,7 +4897,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B80">
         <v>74</v>
       </c>
@@ -4918,7 +4914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B81">
         <v>75</v>
       </c>
@@ -4935,7 +4931,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B82">
         <v>76</v>
       </c>
@@ -4952,7 +4948,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B83">
         <v>77</v>
       </c>
@@ -4969,7 +4965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B84">
         <v>78</v>
       </c>
@@ -4986,7 +4982,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B85">
         <v>79</v>
       </c>
@@ -5003,7 +4999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B86">
         <v>80</v>
       </c>
@@ -5020,7 +5016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B87">
         <v>81</v>
       </c>
@@ -5037,7 +5033,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B88">
         <v>82</v>
       </c>
@@ -5054,7 +5050,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B89">
         <v>83</v>
       </c>
@@ -5071,7 +5067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B90">
         <v>84</v>
       </c>
@@ -5088,7 +5084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B91">
         <v>85</v>
       </c>
@@ -5105,7 +5101,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B92">
         <v>86</v>
       </c>
@@ -5122,7 +5118,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B93">
         <v>87</v>
       </c>
@@ -5139,7 +5135,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B94">
         <v>88</v>
       </c>
@@ -5156,7 +5152,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B95">
         <v>89</v>
       </c>
@@ -5173,7 +5169,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B96">
         <v>90</v>
       </c>
@@ -5190,7 +5186,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B97">
         <v>91</v>
       </c>
@@ -5207,7 +5203,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B98">
         <v>92</v>
       </c>
@@ -5224,7 +5220,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B99">
         <v>93</v>
       </c>
@@ -5241,7 +5237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B100">
         <v>94</v>
       </c>
@@ -5258,7 +5254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B101">
         <v>95</v>
       </c>
@@ -5275,7 +5271,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B102">
         <v>96</v>
       </c>
@@ -5292,7 +5288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B103">
         <v>97</v>
       </c>
@@ -5309,7 +5305,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B104">
         <v>98</v>
       </c>
@@ -5326,7 +5322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B105">
         <v>99</v>
       </c>
@@ -5343,7 +5339,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B106">
         <v>100</v>
       </c>
@@ -5376,26 +5372,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{523B2388-8617-4507-AE93-56CCFC2C84AF}">
   <dimension ref="B2:B7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="97.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:2" ht="228" x14ac:dyDescent="0.45">
       <c r="B2" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:2" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="4" spans="2:2" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="13"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.45">
       <c r="B6" s="48" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.45">
       <c r="B7" s="49" t="s">
         <v>72</v>
       </c>

</xml_diff>